<commit_message>
add workflow top-level metadata
</commit_message>
<xml_diff>
--- a/runs/csmWorkflow-demo/isa.run.xlsx
+++ b/runs/csmWorkflow-demo/isa.run.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="68">
   <si>
     <t>RUN</t>
   </si>
@@ -71,15 +71,27 @@
     <t>Run Technology Type</t>
   </si>
   <si>
+    <t>CWL</t>
+  </si>
+  <si>
     <t>Run Technology Type Term Accession Number</t>
   </si>
   <si>
+    <t>http://purl.obolibrary.org/obo/EDAM_3857</t>
+  </si>
+  <si>
     <t>Run Technology Type Term Source REF</t>
   </si>
   <si>
+    <t>edam</t>
+  </si>
+  <si>
     <t>Run Technology Platform</t>
   </si>
   <si>
+    <t>CWL (EDAM:3857)</t>
+  </si>
+  <si>
     <t>Run File Name</t>
   </si>
   <si>
@@ -92,54 +104,99 @@
     <t>Run Person Last Name</t>
   </si>
   <si>
+    <t>Gitahi</t>
+  </si>
+  <si>
     <t>Run Person First Name</t>
   </si>
   <si>
+    <t>Joseph</t>
+  </si>
+  <si>
     <t>Run Person Mid Initials</t>
   </si>
   <si>
     <t>Run Person Email</t>
   </si>
   <si>
+    <t>joseph.gitahi@tum.de</t>
+  </si>
+  <si>
     <t>Run Person Phone</t>
   </si>
   <si>
+    <t>089 289 22531</t>
+  </si>
+  <si>
     <t>Run Person Fax</t>
   </si>
   <si>
     <t>Run Person Address</t>
   </si>
   <si>
+    <t>Arcisstraße 21, 80333 Münch</t>
+  </si>
+  <si>
     <t>Run Person Affiliation</t>
   </si>
   <si>
+    <t>Technical University of Munich, Chair of Geoinformatics</t>
+  </si>
+  <si>
     <t>Run Person Roles</t>
   </si>
   <si>
+    <t>researcher</t>
+  </si>
+  <si>
     <t>Run Person Roles Term Accession Number</t>
   </si>
   <si>
+    <t>AGRO:00000373</t>
+  </si>
+  <si>
     <t>Run Person Roles Term Source REF</t>
   </si>
   <si>
+    <t>AGRO</t>
+  </si>
+  <si>
+    <t>Comment[ORCID]</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0003-3364-2256</t>
+  </si>
+  <si>
     <t>Input [Data]</t>
   </si>
   <si>
+    <t>Data Format</t>
+  </si>
+  <si>
+    <t>Data Selector Format</t>
+  </si>
+  <si>
     <t>Protocol Uri</t>
   </si>
   <si>
     <t>Output [Data]</t>
   </si>
   <si>
+    <t xml:space="preserve">Data Format </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Selector Format </t>
+  </si>
+  <si>
     <t>geojson</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>./workflows/csmWorkflow/workflow.cwl</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>longitude</t>
   </si>
   <si>
@@ -167,10 +224,13 @@
     <t>ndvi_file</t>
   </si>
   <si>
-    <t>phenology_results_csv</t>
+    <t>ndvi_timeseries.csv</t>
   </si>
   <si>
     <t>geojson_file</t>
+  </si>
+  <si>
+    <t>field_location.geojson</t>
   </si>
   <si>
     <t>phenology_results_png</t>
@@ -232,16 +292,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="annotationTable0" displayName="annotationTable0" ref="A1:C8" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A1:C8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="annotationTable0" displayName="annotationTable0" ref="A1:G8" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A1:G8">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="3">
+  <tableColumns count="7">
     <tableColumn id="1" name="Input [Data]" totalsRowLabel="Total"/>
-    <tableColumn id="2" name="Protocol Uri" totalsRowFunction="none"/>
-    <tableColumn id="3" name="Output [Data]" totalsRowFunction="none"/>
+    <tableColumn id="2" name="Data Format" totalsRowFunction="none"/>
+    <tableColumn id="3" name="Data Selector Format" totalsRowFunction="none"/>
+    <tableColumn id="4" name="Protocol Uri" totalsRowFunction="none"/>
+    <tableColumn id="5" name="Output [Data]" totalsRowFunction="none"/>
+    <tableColumn id="6" name="Data Format " totalsRowFunction="none"/>
+    <tableColumn id="7" name="Data Selector Format " totalsRowFunction="none"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -608,7 +676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -660,92 +728,139 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>17</v>
+      </c>
+      <c r="B12" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="B15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>24</v>
+      </c>
+      <c r="B16" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>22</v>
+        <v>29</v>
+      </c>
+      <c r="B19" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+      <c r="B21" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="B22" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="B23" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="B24" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>40</v>
+      </c>
+      <c r="B25" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B26" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -756,95 +871,191 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="B1" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="C1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+      <c r="D1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="D2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="D3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="D4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="D5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="D6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="B7" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="D7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="B8" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>52</v>
+      </c>
+      <c r="D8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F8" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -863,46 +1074,46 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="B1" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="C1" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -921,57 +1132,57 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="B1" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="C1" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="C4" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -990,46 +1201,46 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="B1" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="C1" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1048,46 +1259,46 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="B1" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="C1" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
complete csmWorkflow and run definitions
- Extend workflow.cwl to all 18 steps (fetch-ndvi through plot-results)
- Update run.cwl to match workflow.cwl inputs, steps and outputs
</commit_message>
<xml_diff>
--- a/runs/csmWorkflow-demo/isa.run.xlsx
+++ b/runs/csmWorkflow-demo/isa.run.xlsx
@@ -10,13 +10,15 @@
     <sheet sheetId="4" name="P2-GrowthStageExtraction" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="P3-DataAcquisition" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="P4-DataIntegration" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="P5-DSSATSimulation" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="NewTable1" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="68">
   <si>
     <t>RUN</t>
   </si>
@@ -365,6 +367,22 @@
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" name="annotationTable4" displayName="annotationTable4" ref="A1:C4" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A1:C4">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Input [Sample Name]" totalsRowLabel="Total"/>
+    <tableColumn id="2" name="Protocol REF" totalsRowFunction="none"/>
+    <tableColumn id="3" name="Output [Sample Name]" totalsRowFunction="none"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" name="annotationTable5" displayName="annotationTable5" ref="A1:C4" totalsRowShown="1" headerRowCount="1">
   <autoFilter ref="A1:C4">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1308,4 +1326,72 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>